<commit_message>
feat: handle empty sync fields and implement 2-way reload sync with sync_delete
</commit_message>
<xml_diff>
--- a/File_lưu.xlsx
+++ b/File_lưu.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2256" yWindow="1020" windowWidth="18576" windowHeight="8952" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Thang 03" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Nghiệp đoàn" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Chủ sử dụng" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Phái Cử" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thang 03" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nghiệp đoàn" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chủ sử dụng" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phái Cử" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: candidate form template & importer, remove gsheet, dark mode, manual date input
</commit_message>
<xml_diff>
--- a/File_lưu.xlsx
+++ b/File_lưu.xlsx
@@ -2,55 +2,40 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2256" yWindow="1020" windowWidth="18576" windowHeight="8952" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thang 03" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thang 08" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nghiệp đoàn" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chủ sử dụng" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phái Cử" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Arial"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="14"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="16"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -58,7 +43,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,20 +52,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.3999755851924192"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="001E3A5F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.7999816888943144"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.3999755851924192"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="00F0F4FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -89,7 +66,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -97,43 +74,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00AAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -216,44 +193,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -280,32 +257,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -332,24 +291,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -361,142 +302,166 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
@@ -506,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BH5"/>
+  <dimension ref="A1:BH19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -572,302 +537,302 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B1" s="14" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>MA HO SO</t>
         </is>
       </c>
-      <c r="C1" s="14" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>TEN VNM</t>
         </is>
       </c>
-      <c r="D1" s="14" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>TEN ENG</t>
         </is>
       </c>
-      <c r="E1" s="14" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>TEN PHIEN AM</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>GIOI TINH JPN</t>
         </is>
       </c>
-      <c r="G1" s="14" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>SO CAN CUOC</t>
         </is>
       </c>
-      <c r="H1" s="14" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>NGAY CAP CAN CUOC VNM</t>
         </is>
       </c>
-      <c r="I1" s="14" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>NGAY CAP CAN CUOC JPN</t>
         </is>
       </c>
-      <c r="J1" s="14" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>NOI CAP CAN CUOC VNM</t>
         </is>
       </c>
-      <c r="K1" s="14" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>NOI CAP CAN CUOC JPN</t>
         </is>
       </c>
-      <c r="L1" s="14" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>SO HO CHIEU</t>
         </is>
       </c>
-      <c r="M1" s="14" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>NGAY CAP HO CHIEU VNM</t>
         </is>
       </c>
-      <c r="N1" s="14" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>NGAY CAP HO CHIEU JPN</t>
         </is>
       </c>
-      <c r="O1" s="14" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>NOI CAP HO CHIEU VNM</t>
         </is>
       </c>
-      <c r="P1" s="14" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>NOI CAP HO CHIEU JPN</t>
         </is>
       </c>
-      <c r="Q1" s="14" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>NAM SINH VNM</t>
         </is>
       </c>
-      <c r="R1" s="14" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>NAM SINH JPN</t>
         </is>
       </c>
-      <c r="S1" s="14" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>TINH TRANG HON NHAN</t>
         </is>
       </c>
-      <c r="T1" s="14" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>CO CON</t>
         </is>
       </c>
-      <c r="U1" s="14" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>DIA CHI VNM</t>
         </is>
       </c>
-      <c r="V1" s="14" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>DIA CHI JPN</t>
         </is>
       </c>
-      <c r="W1" s="14" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>NOI SINH VNM</t>
         </is>
       </c>
-      <c r="X1" s="14" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>NOI SINH JPN</t>
         </is>
       </c>
-      <c r="Y1" s="14" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>NGUOI GIAM HO VNM</t>
         </is>
       </c>
-      <c r="Z1" s="14" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>NGUOI GIAM HO JPN</t>
         </is>
       </c>
-      <c r="AA1" s="14" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>DIA CHI NGUOI GIAM HO VNM</t>
         </is>
       </c>
-      <c r="AB1" s="14" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>DIA CHI NGUOI GIAM HO JPN</t>
         </is>
       </c>
-      <c r="AC1" s="14" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>SDT NGUOI GIAM HO</t>
         </is>
       </c>
-      <c r="AD1" s="14" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>TRUONG HOC 1 VNM</t>
         </is>
       </c>
-      <c r="AE1" s="14" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>TRUONG HOC 1 JPN</t>
         </is>
       </c>
-      <c r="AF1" s="14" t="inlineStr">
+      <c r="AF1" s="4" t="inlineStr">
         <is>
           <t>TRUONG HOC 2 VNM</t>
         </is>
       </c>
-      <c r="AG1" s="14" t="inlineStr">
+      <c r="AG1" s="4" t="inlineStr">
         <is>
           <t>TRUONG HOC 2 JPN</t>
         </is>
       </c>
-      <c r="AH1" s="14" t="inlineStr">
+      <c r="AH1" s="4" t="inlineStr">
         <is>
           <t>TRUONG HOC 3 VNM</t>
         </is>
       </c>
-      <c r="AI1" s="14" t="inlineStr">
+      <c r="AI1" s="4" t="inlineStr">
         <is>
           <t>TRUONG HOC 3 JPN</t>
         </is>
       </c>
-      <c r="AJ1" s="14" t="inlineStr">
+      <c r="AJ1" s="4" t="inlineStr">
         <is>
           <t>CONG TY 1 VNM</t>
         </is>
       </c>
-      <c r="AK1" s="14" t="inlineStr">
+      <c r="AK1" s="4" t="inlineStr">
         <is>
           <t>CONG TY 1 JPN</t>
         </is>
       </c>
-      <c r="AL1" s="14" t="inlineStr">
+      <c r="AL1" s="4" t="inlineStr">
         <is>
           <t>CONG TY 2 VNM</t>
         </is>
       </c>
-      <c r="AM1" s="14" t="inlineStr">
+      <c r="AM1" s="4" t="inlineStr">
         <is>
           <t>CONG TY 2 JPN</t>
         </is>
       </c>
-      <c r="AN1" s="14" t="inlineStr">
+      <c r="AN1" s="4" t="inlineStr">
         <is>
           <t>CONG TY 3 VNM</t>
         </is>
       </c>
-      <c r="AO1" s="14" t="inlineStr">
+      <c r="AO1" s="4" t="inlineStr">
         <is>
           <t>CONG TY 3 JPN</t>
         </is>
       </c>
-      <c r="AP1" s="14" t="inlineStr">
+      <c r="AP1" s="4" t="inlineStr">
         <is>
           <t>LINH VUC THUC TAP VNM</t>
         </is>
       </c>
-      <c r="AQ1" s="14" t="inlineStr">
+      <c r="AQ1" s="4" t="inlineStr">
         <is>
           <t>LINH VUC THUC TAP JPN</t>
         </is>
       </c>
-      <c r="AR1" s="14" t="inlineStr">
+      <c r="AR1" s="4" t="inlineStr">
         <is>
           <t>TOM TAT KN JPN</t>
         </is>
       </c>
-      <c r="AS1" s="14" t="inlineStr">
+      <c r="AS1" s="4" t="inlineStr">
         <is>
           <t>TOM TAT KN VNM</t>
         </is>
       </c>
-      <c r="AT1" s="14" t="inlineStr">
+      <c r="AT1" s="4" t="inlineStr">
         <is>
           <t>NGHIEP DOAN VNM</t>
         </is>
       </c>
-      <c r="AU1" s="14" t="inlineStr">
+      <c r="AU1" s="4" t="inlineStr">
         <is>
           <t>NGHIEP DOAN JPN</t>
         </is>
       </c>
-      <c r="AV1" s="14" t="inlineStr">
+      <c r="AV1" s="4" t="inlineStr">
         <is>
           <t>DC NGHIEP DOAN VNM</t>
         </is>
       </c>
-      <c r="AW1" s="14" t="inlineStr">
+      <c r="AW1" s="4" t="inlineStr">
         <is>
           <t>DC NGHIEP DOAN JPN</t>
         </is>
       </c>
-      <c r="AX1" s="14" t="inlineStr">
+      <c r="AX1" s="4" t="inlineStr">
         <is>
           <t>ND NGHIEP DOAN VNM</t>
         </is>
       </c>
-      <c r="AY1" s="14" t="inlineStr">
+      <c r="AY1" s="4" t="inlineStr">
         <is>
           <t>ND NGHIEP DOAN JPN</t>
         </is>
       </c>
-      <c r="AZ1" s="14" t="inlineStr">
+      <c r="AZ1" s="4" t="inlineStr">
         <is>
           <t>CONG TY TIEP NHAN VNM</t>
         </is>
       </c>
-      <c r="BA1" s="14" t="inlineStr">
+      <c r="BA1" s="4" t="inlineStr">
         <is>
           <t>CONG TY TIEP NHAN JPN</t>
         </is>
       </c>
-      <c r="BB1" s="14" t="inlineStr">
+      <c r="BB1" s="4" t="inlineStr">
         <is>
           <t>DC CONG TY TIEP NHAN VNM</t>
         </is>
       </c>
-      <c r="BC1" s="14" t="inlineStr">
+      <c r="BC1" s="4" t="inlineStr">
         <is>
           <t>DC CONG TY TIEP NHAN JPN</t>
         </is>
       </c>
-      <c r="BD1" s="14" t="inlineStr">
+      <c r="BD1" s="4" t="inlineStr">
         <is>
           <t>ND CONG TY TIEP NHAN VNM</t>
         </is>
       </c>
-      <c r="BE1" s="14" t="inlineStr">
+      <c r="BE1" s="4" t="inlineStr">
         <is>
           <t>ND CONG TY TIEP NHAN JPN</t>
         </is>
       </c>
-      <c r="BF1" s="14" t="inlineStr">
+      <c r="BF1" s="4" t="inlineStr">
         <is>
           <t>CONG TY PHAI CU VNM</t>
         </is>
       </c>
-      <c r="BG1" s="14" t="inlineStr">
+      <c r="BG1" s="4" t="inlineStr">
         <is>
           <t>ND CONG TY PHAI CU VNM</t>
         </is>
       </c>
-      <c r="BH1" s="14" t="inlineStr">
+      <c r="BH1" s="4" t="inlineStr">
         <is>
           <t>SO DIEN THOAI</t>
         </is>
@@ -1886,6 +1851,1886 @@
       <c r="BH5" t="inlineStr">
         <is>
           <t>0398930443</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TTS-005</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Updated</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NGUYEN VAN TEST</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>グエン ヴァン テスト</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>000111222333</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>01/01/2020</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>15/01/2000</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2000年01月15日</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>0911111111</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Trường THPT ABC</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="inlineStr"/>
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr"/>
+      <c r="AJ6" t="inlineStr"/>
+      <c r="AK6" t="inlineStr"/>
+      <c r="AL6" t="inlineStr"/>
+      <c r="AM6" t="inlineStr"/>
+      <c r="AN6" t="inlineStr"/>
+      <c r="AO6" t="inlineStr"/>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AR6" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AS6" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr"/>
+      <c r="BB6" t="inlineStr"/>
+      <c r="BC6" t="inlineStr"/>
+      <c r="BD6" t="inlineStr"/>
+      <c r="BE6" t="inlineStr"/>
+      <c r="BF6" t="inlineStr"/>
+      <c r="BG6" t="inlineStr"/>
+      <c r="BH6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TTS-006</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Auto Code Test</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="inlineStr"/>
+      <c r="AH7" t="inlineStr"/>
+      <c r="AI7" t="inlineStr"/>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
+      <c r="AL7" t="inlineStr"/>
+      <c r="AM7" t="inlineStr"/>
+      <c r="AN7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr"/>
+      <c r="AP7" t="inlineStr"/>
+      <c r="AQ7" t="inlineStr"/>
+      <c r="AR7" t="inlineStr"/>
+      <c r="AS7" t="inlineStr"/>
+      <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr"/>
+      <c r="BB7" t="inlineStr"/>
+      <c r="BC7" t="inlineStr"/>
+      <c r="BD7" t="inlineStr"/>
+      <c r="BE7" t="inlineStr"/>
+      <c r="BF7" t="inlineStr"/>
+      <c r="BG7" t="inlineStr"/>
+      <c r="BH7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TTS-007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Trần Thị Full</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TRAN THI FULL</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>チャン ティ フル</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>012345678901</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>10/05/2021</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>B1234567</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>15/03/2022</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>20/06/1998</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1998年06月20日</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Độc thân</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>ハノイ市 フエ通り123</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>ハノイ</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>Trần Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>チャン ヴァン チャ</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr"/>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>ハノイ高校</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>ハノイ工科大学</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr"/>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>ABC縫製会社</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="inlineStr"/>
+      <c r="AN8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr"/>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr"/>
+      <c r="AY8" t="inlineStr"/>
+      <c r="AZ8" t="inlineStr"/>
+      <c r="BA8" t="inlineStr"/>
+      <c r="BB8" t="inlineStr"/>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TTS-008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Updated</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>NGUYEN VAN TEST</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>グエン ヴァン テスト</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>000111222333</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>01/01/2020</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>15/01/2000</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2000年01月15日</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr"/>
+      <c r="AB9" t="inlineStr"/>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>0911111111</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Trường THPT ABC</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="inlineStr"/>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr"/>
+      <c r="AN9" t="inlineStr"/>
+      <c r="AO9" t="inlineStr"/>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr"/>
+      <c r="BB9" t="inlineStr"/>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TTS-009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Auto Code Test</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
+      <c r="Z10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
+      <c r="AC10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="inlineStr"/>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="inlineStr"/>
+      <c r="AN10" t="inlineStr"/>
+      <c r="AO10" t="inlineStr"/>
+      <c r="AP10" t="inlineStr"/>
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr"/>
+      <c r="AS10" t="inlineStr"/>
+      <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr"/>
+      <c r="BB10" t="inlineStr"/>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TTS-010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Trần Thị Full</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TRAN THI FULL</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>チャン ティ フル</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>012345678901</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>10/05/2021</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>B1234567</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>15/03/2022</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>20/06/1998</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1998年06月20日</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Độc thân</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>ハノイ市 フエ通り123</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>ハノイ</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Trần Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>チャン ヴァン チャ</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr"/>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>ハノイ高校</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>ハノイ工科大学</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr"/>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>ABC縫製会社</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="inlineStr"/>
+      <c r="AN11" t="inlineStr"/>
+      <c r="AO11" t="inlineStr"/>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr"/>
+      <c r="AY11" t="inlineStr"/>
+      <c r="AZ11" t="inlineStr"/>
+      <c r="BA11" t="inlineStr"/>
+      <c r="BB11" t="inlineStr"/>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
+      <c r="BG11" t="inlineStr"/>
+      <c r="BH11" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TTS-012</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Auto Code Test</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="inlineStr"/>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
+      <c r="BB12" t="inlineStr"/>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr"/>
+      <c r="BG12" t="inlineStr"/>
+      <c r="BH12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TTS-013</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Trần Thị Full</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TRAN THI FULL</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>チャン ティ フル</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>012345678901</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>10/05/2021</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>B1234567</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>15/03/2022</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>20/06/1998</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1998年06月20日</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Độc thân</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>ハノイ市 フエ通り123</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>ハノイ</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Trần Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>チャン ヴァン チャ</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>THPT Chuyên Hà Nội</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>ハノイ高校</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Đại học Bách Khoa Hà Nội</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>ハノイ工科大学</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>Công ty May ABC</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>ABC縫製会社</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr"/>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TTS-014</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Updated</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>NGUYEN VAN TEST</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>グエン ヴァン テスト</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>000111222333</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>01/01/2020</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>15/01/2000</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>2000年01月15日</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>0911111111</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Trường THPT ABC</t>
+        </is>
+      </c>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+      <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr"/>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="inlineStr"/>
+      <c r="BH14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TTS-015</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Auto Code Test</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr"/>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr"/>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="inlineStr"/>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="inlineStr"/>
+      <c r="AN15" t="inlineStr"/>
+      <c r="AO15" t="inlineStr"/>
+      <c r="AP15" t="inlineStr"/>
+      <c r="AQ15" t="inlineStr"/>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
+      <c r="AZ15" t="inlineStr"/>
+      <c r="BA15" t="inlineStr"/>
+      <c r="BB15" t="inlineStr"/>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr"/>
+      <c r="BH15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TTS-016</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Trần Thị Full</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TRAN THI FULL</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>チャン ティ フル</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>012345678901</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>10/05/2021</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>B1234567</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>15/03/2022</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>20/06/1998</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1998年06月20日</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Độc thân</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>ハノイ市 フエ通り123</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>ハノイ</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>Trần Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>チャン ヴァン チャ</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>THPT Chuyên Hà Nội</t>
+        </is>
+      </c>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>ハノイ高校</t>
+        </is>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Đại học Bách Khoa Hà Nội</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>ハノイ工科大学</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr">
+        <is>
+          <t>Công ty May ABC</t>
+        </is>
+      </c>
+      <c r="AK16" t="inlineStr">
+        <is>
+          <t>ABC縫製会社</t>
+        </is>
+      </c>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr"/>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr"/>
+      <c r="BH16" t="inlineStr">
+        <is>
+          <t>0912345678</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TTS-017</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Updated</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NGUYEN VAN TEST</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>グエン ヴァン テスト</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Nam</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>000111222333</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>01/01/2020</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>15/01/2000</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>2000年01月15日</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>0911111111</t>
+        </is>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Trường THPT ABC</t>
+        </is>
+      </c>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr"/>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>２年</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>2 năm</t>
+        </is>
+      </c>
+      <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+      <c r="AZ17" t="inlineStr"/>
+      <c r="BA17" t="inlineStr"/>
+      <c r="BB17" t="inlineStr"/>
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr"/>
+      <c r="BG17" t="inlineStr"/>
+      <c r="BH17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>TTS-018</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Auto Code Test</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr"/>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
+      <c r="BB18" t="inlineStr"/>
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr"/>
+      <c r="BG18" t="inlineStr"/>
+      <c r="BH18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TTS-019</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Trần Thị Full</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TRAN THI FULL</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>チャン ティ フル</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Nữ</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>012345678901</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>10/05/2021</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>B1234567</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>15/03/2022</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>20/06/1998</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1998年06月20日</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Độc thân</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>Không</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>ハノイ市 フエ通り123</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Hà Nội</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>ハノイ</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>Trần Văn Cha</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>チャン ヴァン チャ</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>123 Phố Huế, Hà Nội</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr"/>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>0987654321</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>THPT Chuyên Hà Nội</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>ハノイ高校</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>Đại học Bách Khoa Hà Nội</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>ハノイ工科大学</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>Công ty May ABC</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>ABC縫製会社</t>
+        </is>
+      </c>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="inlineStr"/>
+      <c r="AN19" t="inlineStr"/>
+      <c r="AO19" t="inlineStr"/>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>３年縫製</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>3 năm may mặc</t>
+        </is>
+      </c>
+      <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr"/>
+      <c r="BB19" t="inlineStr"/>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr">
+        <is>
+          <t>0912345678</t>
         </is>
       </c>
     </row>
@@ -1900,133 +3745,135 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="10.796875" defaultRowHeight="17.4"/>
+  <dimension ref="A2:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.796875" customWidth="1" style="1" min="1" max="1"/>
-    <col width="49.5" bestFit="1" customWidth="1" style="1" min="2" max="2"/>
-    <col width="37" bestFit="1" customWidth="1" style="1" min="3" max="3"/>
-    <col width="25.5" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
-    <col width="26" bestFit="1" customWidth="1" style="1" min="5" max="5"/>
-    <col width="24.5" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
-    <col width="23.796875" bestFit="1" customWidth="1" style="1" min="7" max="7"/>
-    <col width="16.5" bestFit="1" customWidth="1" style="4" min="8" max="8"/>
-    <col width="10.796875" customWidth="1" style="1" min="9" max="16384"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="2" ht="40.8" customFormat="1" customHeight="1" s="5">
-      <c r="B2" s="5" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>TEN ND VNM</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>TEN ND JPN</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>CHU TICH ND VNM</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>CHU TICH ND JPN</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>D/C NGHIEP DOAN VNM</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>D/C NGHIEP DOAN JPN</t>
         </is>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>SDT JAPAN</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="1" t="inlineStr">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Nghiệp đoàn kinh doanh nông nghiệp Maruko</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>マルコ・アグリビジネス協同組合</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>Kobayashi Kouji</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>KOBAYASHI KOUJI</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>小林　浩治</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>1387-53 Tokujuku, Thành phố Hokota, Tỉnh Ibaraki</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>茨城県鉾田市徳宿1387-53</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>0291-36-5400</t>
-        </is>
-      </c>
+      <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="B4" s="1" t="inlineStr">
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Nghiệp đoàn YS Support Kyodo Kumiai</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>イースサポート協同組合</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Nguyễn Thị Thuý Hằng</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Nguyen Thi Thuy Hang</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Aichi-ken, Nagoya-shi, Minami-ku, Miyoshi-cho, 6 Chome 8 Banchi 37</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>愛知県名古屋市南区三吉町６丁目８番地の37</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">052-880-6344               </t>
-        </is>
-      </c>
+      <c r="H4" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2036,222 +3883,170 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H5"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="10.796875" defaultRowHeight="17.4"/>
+  <dimension ref="A2:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10.796875" customWidth="1" style="1" min="1" max="1"/>
-    <col width="28.796875" customWidth="1" style="1" min="2" max="2"/>
-    <col width="26.5" customWidth="1" style="1" min="3" max="3"/>
-    <col width="19.796875" customWidth="1" style="1" min="4" max="4"/>
-    <col width="19.5" customWidth="1" style="1" min="5" max="5"/>
-    <col width="20.296875" bestFit="1" customWidth="1" style="1" min="6" max="6"/>
-    <col width="20.5" customWidth="1" style="1" min="7" max="7"/>
-    <col width="10.796875" customWidth="1" style="1" min="8" max="16384"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1"/>
-    <row r="2" ht="60" customFormat="1" customHeight="1" s="2">
-      <c r="B2" s="2" t="inlineStr">
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>TEN TO CHUC THUC TAP VNM</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>TEN TO CHUC THUC TAP JPN</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>TEN GIAM DOC VNM</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>TEN GD JPN</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>D/C THUC TAP VNM</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>D/C THUC TAP JPN</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>SO DIEN THOAI</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="B3" s="1" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>KITAYAMA YASUSHI</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>北山 靖</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>KITAYAMA YASUSHI</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>北山 靖</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">221-172 Funaki Hokota-shi Ibarki-ken </t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>221-172 Funaki Hokota-shi Ibarki-ken</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>茨城県鉾田市舟木 221-172</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>0291-36-2189</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>CTY CP KITAGAWA KOUMUTEN</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>株式会社北川工務店</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>KITAGAWA HARUMASA</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
-        <is>
-          <t>北川　晴将</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Gifu-ken, Hashima-shi, Masaki-cho, Sugakomatsu 459</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr">
-        <is>
-          <t>岐阜県羽島市正木町須賀小松459番地</t>
-        </is>
-      </c>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>058-392-5035</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="1" t="inlineStr">
-        <is>
-          <t>CTY TNHH SAWADAJUKI</t>
-        </is>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>有限会社澤田重機</t>
-        </is>
-      </c>
-      <c r="D5" s="1" t="inlineStr">
-        <is>
-          <t>SAWADA SHIGEMI</t>
-        </is>
-      </c>
-      <c r="E5" s="1" t="inlineStr">
-        <is>
-          <t>澤田　茂美</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr">
-        <is>
-          <t>Gifu-ken, Ghifu-shi, Noishiki 6 chome 8-14</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr">
-        <is>
-          <t>岐阜県岐阜市野一色六丁目8番14号</t>
-        </is>
-      </c>
-      <c r="H5" s="1" t="inlineStr">
-        <is>
-          <t>058-247-1700</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1"/>
-    <row r="7" ht="30" customHeight="1"/>
-    <row r="8" ht="30" customHeight="1"/>
-    <row r="9" ht="30" customHeight="1"/>
-    <row r="10" ht="30" customHeight="1"/>
-    <row r="11" ht="30" customHeight="1"/>
-    <row r="12" ht="30" customHeight="1"/>
-    <row r="13" ht="30" customHeight="1"/>
-    <row r="14" ht="30" customHeight="1"/>
-    <row r="15" ht="30" customHeight="1"/>
-    <row r="16" ht="30" customHeight="1"/>
-    <row r="17" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="18" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="19" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="20" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="21" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="22" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="23" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="24" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="25" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="26" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="27" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="28" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="29" ht="30" customFormat="1" customHeight="1" s="1"/>
-    <row r="30" ht="30" customFormat="1" customHeight="1" s="1"/>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B3:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
-  <sheetData>
-    <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">送出機関：TRUONG SON TRADING SERVICE AND LABOR EXPORT JOINT STOCK COMPANY (COOPIMEX JSC) </t>
-        </is>
-      </c>
+      <c r="H3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>代表者：NGUYEN THI HOA</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>CTY CP KITAGAWA KOUMUTEN</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>株式会社北川工務店</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>KITAGAWA HARUMASA</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>北川　晴将</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Gifu-ken, Hashima-shi, Masaki-cho, Sugakomatsu 459</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>岐阜県羽島市正木町須賀小松459番地</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>CTY TNHH SAWADAJUKI</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>有限会社澤田重機</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>SAWADA SHIGEMI</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>澤田　茂美</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Gifuken Gifushi Noishiki 6chome 8-14</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>岐阜県岐阜市野一色六丁目8番14号</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>